<commit_message>
Automatiza 1 arquivo(s) de processos no painel
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG + ECO HIBRIDO LADO MENOR.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG + ECO HIBRIDO LADO MENOR.xlsx
@@ -323,7 +323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -1534,8 +1534,9 @@
           <t>20X20X1,50MM Nest 1</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>0.331</v>
+      <c r="D43">
+        <f>E43/1000</f>
+        <v/>
       </c>
       <c r="E43" t="n">
         <v>331</v>
@@ -1562,8 +1563,9 @@
           <t>20X20X1,50MM Nest 2</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>0.001</v>
+      <c r="D44">
+        <f>E44/1000</f>
+        <v/>
       </c>
       <c r="E44" t="n">
         <v>1</v>
@@ -1590,8 +1592,9 @@
           <t>20X20X1,50MM Nest 3</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>0.001</v>
+      <c r="D45">
+        <f>E45/1000</f>
+        <v/>
       </c>
       <c r="E45" t="n">
         <v>1</v>
@@ -1618,8 +1621,9 @@
           <t>20X20X1,50MM Nest 4</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>0.332</v>
+      <c r="D46">
+        <f>E46/1000</f>
+        <v/>
       </c>
       <c r="E46" t="n">
         <v>332</v>
@@ -1646,8 +1650,9 @@
           <t>20X20X1,50MM Nest 5</t>
         </is>
       </c>
-      <c r="D47" t="n">
-        <v>0.332</v>
+      <c r="D47">
+        <f>E47/1000</f>
+        <v/>
       </c>
       <c r="E47" t="n">
         <v>332</v>
@@ -1674,8 +1679,9 @@
           <t>20X20X1,50MM Nest 6</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>0.332</v>
+      <c r="D48">
+        <f>E48/1000</f>
+        <v/>
       </c>
       <c r="E48" t="n">
         <v>332</v>
@@ -1702,8 +1708,9 @@
           <t>20X20X1,50MM Nest 7</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>0.001</v>
+      <c r="D49">
+        <f>E49/1000</f>
+        <v/>
       </c>
       <c r="E49" t="n">
         <v>1</v>
@@ -2485,7 +2492,7 @@
         </is>
       </c>
       <c r="D76">
-        <f>E76/1700</f>
+        <f>E76/1000</f>
         <v/>
       </c>
       <c r="E76" t="n">
@@ -2514,11 +2521,11 @@
         </is>
       </c>
       <c r="D77">
-        <f>E77/1700</f>
+        <f>E77/1000</f>
         <v/>
       </c>
       <c r="E77" t="n">
-        <v>130</v>
+        <v>99</v>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
@@ -2543,11 +2550,11 @@
         </is>
       </c>
       <c r="D78">
-        <f>E78/1700</f>
+        <f>E78/1000</f>
         <v/>
       </c>
       <c r="E78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
@@ -2572,11 +2579,11 @@
         </is>
       </c>
       <c r="D79">
-        <f>E79/1700</f>
+        <f>E79/1000</f>
         <v/>
       </c>
       <c r="E79" t="n">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
@@ -2601,11 +2608,11 @@
         </is>
       </c>
       <c r="D80">
-        <f>E80/1700</f>
+        <f>E80/1000</f>
         <v/>
       </c>
       <c r="E80" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
@@ -2630,7 +2637,7 @@
         </is>
       </c>
       <c r="D81">
-        <f>E81/1700</f>
+        <f>E81/1000</f>
         <v/>
       </c>
       <c r="E81" t="n">
@@ -2659,11 +2666,11 @@
         </is>
       </c>
       <c r="D82">
-        <f>E82/1700</f>
+        <f>E82/1000</f>
         <v/>
       </c>
       <c r="E82" t="n">
-        <v>221</v>
+        <v>5</v>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
@@ -2688,7 +2695,7 @@
         </is>
       </c>
       <c r="D83">
-        <f>E83/1700</f>
+        <f>E83/1000</f>
         <v/>
       </c>
       <c r="E83" t="n">
@@ -2708,24 +2715,23 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Serra</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2,65 Nest 9</t>
-        </is>
-      </c>
-      <c r="D84">
-        <f>E84/1700</f>
-        <v/>
+          <t>Tubo Bdj 433 MM</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>5</v>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>5000</v>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>000345</t>
+          <t>000379</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2748,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Tubo Bdj 433 MM</t>
+          <t>Tubo Bdj 493 MM</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2753,7 +2759,7 @@
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>000379</t>
+          <t>000380</t>
         </is>
       </c>
     </row>
@@ -2765,23 +2771,23 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Serra</t>
+          <t>Dobradeira de Arames</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Tubo Bdj 493 MM</t>
+          <t>Arame Toldo Lateral</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E86" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>000380</t>
+          <t>001439</t>
         </is>
       </c>
     </row>
@@ -2798,18 +2804,18 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Arame Toldo Lateral</t>
+          <t>Arame Toldo Trecho Reto</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E87" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>001439</t>
+          <t>001440</t>
         </is>
       </c>
     </row>
@@ -2821,23 +2827,23 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Dobradeira de Arames</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Arame Toldo Trecho Reto</t>
+          <t>J 1732 mm</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E88" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>001440</t>
+          <t>000346</t>
         </is>
       </c>
     </row>
@@ -2854,18 +2860,18 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>J 1732 mm</t>
+          <t>J 333 mm</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E89" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>000346</t>
+          <t>000347</t>
         </is>
       </c>
     </row>
@@ -2882,18 +2888,18 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>J 333 mm</t>
+          <t>J 1028 mm</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>000347</t>
+          <t>000348</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2916,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>J 1028 mm</t>
+          <t>Fechamento Saia</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2921,7 +2927,7 @@
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>000348</t>
+          <t>000349</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2944,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Fechamento Saia</t>
+          <t>Fechamento Parachoque Móvel</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2949,7 +2955,7 @@
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>000349</t>
+          <t>000350</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2972,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Fechamento Parachoque Móvel</t>
+          <t>Chapa Frontal Testeira</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -2977,7 +2983,7 @@
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>000350</t>
+          <t>000351</t>
         </is>
       </c>
     </row>
@@ -2994,7 +3000,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Chapa Frontal Testeira</t>
+          <t>Chapa Central Fixação Toldo</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -3005,7 +3011,7 @@
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>000351</t>
+          <t>000352</t>
         </is>
       </c>
     </row>
@@ -3022,18 +3028,18 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Chapa Central Fixação Toldo</t>
+          <t>Encaixe Parachoque Direito</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E95" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>000352</t>
+          <t>000353</t>
         </is>
       </c>
     </row>
@@ -3050,18 +3056,18 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Encaixe Parachoque Direito</t>
+          <t>Encaixe Parachoque Esquerda</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E96" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>000353</t>
+          <t>000354</t>
         </is>
       </c>
     </row>
@@ -3078,18 +3084,18 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Encaixe Parachoque Esquerda</t>
+          <t>Bdj Esquerda Amassamento</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E97" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>000354</t>
+          <t>000355</t>
         </is>
       </c>
     </row>
@@ -3106,7 +3112,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Amassamento</t>
+          <t>Bdj Esquerda Dobra</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -3117,7 +3123,7 @@
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>000355</t>
+          <t>000356</t>
         </is>
       </c>
     </row>
@@ -3134,7 +3140,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Dobra</t>
+          <t>Bdj Direita Amassamento</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3145,7 +3151,7 @@
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>000356</t>
+          <t>000357</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3168,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Bdj Direita Amassamento</t>
+          <t>Bdj Direita Dobra</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -3173,7 +3179,7 @@
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>000357</t>
+          <t>000358</t>
         </is>
       </c>
     </row>
@@ -3190,18 +3196,18 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Bdj Direita Dobra</t>
+          <t>Bdj Esquerda Base Amassamento</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E101" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>000358</t>
+          <t>000359</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3224,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Base Amassamento</t>
+          <t>Bdj Esquerda Base Dobra</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3229,7 +3235,7 @@
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>000359</t>
+          <t>000360</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3252,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Base Dobra</t>
+          <t>Bdj Direita Base Amassamento</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -3257,7 +3263,7 @@
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>000360</t>
+          <t>000361</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3280,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Bdj Direita Base Amassamento</t>
+          <t>Bdj Direita Base Dobra</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3285,7 +3291,7 @@
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>000361</t>
+          <t>000362</t>
         </is>
       </c>
     </row>
@@ -3302,18 +3308,18 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Bdj Direita Base Dobra</t>
+          <t>Chapa Gancho Pallet</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E105" t="n">
         <v>1000</v>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>000362</t>
+          <t>000363</t>
         </is>
       </c>
     </row>
@@ -3325,23 +3331,23 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Chapa Gancho Pallet</t>
+          <t>Lateral Esquerda Tubular</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E106" t="n">
         <v>1000</v>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>000363</t>
+          <t>000364</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3364,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Lateral Esquerda Tubular</t>
+          <t>Lateral Direita Tubular</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3369,7 +3375,7 @@
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>000364</t>
+          <t>000365</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3392,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Lateral Direita Tubular</t>
+          <t>Lateral Esquerda Chaparia + Triângulo 2,65</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3397,7 +3403,7 @@
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>000365</t>
+          <t>000366</t>
         </is>
       </c>
     </row>
@@ -3414,7 +3420,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Lateral Esquerda Chaparia + Triângulo 2,65</t>
+          <t>Lateral Direita Chaparia + Triângulo 2,65</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3425,7 +3431,7 @@
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>000366</t>
+          <t>000367</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3448,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Lateral Direita Chaparia + Triângulo 2,65</t>
+          <t>Lateral Esquerda Arruela Quadrada 2,65</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3453,7 +3459,7 @@
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>000367</t>
+          <t>000368</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3476,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Lateral Esquerda Arruela Quadrada 2,65</t>
+          <t>Lateral Direita Arruela Quadrada 2,65</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3481,7 +3487,7 @@
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>000368</t>
+          <t>000369</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3504,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Lateral Direita Arruela Quadrada 2,65</t>
+          <t>Quadro Cremalheira</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3509,7 +3515,7 @@
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>000369</t>
+          <t>000386</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3532,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Quadro Cremalheira</t>
+          <t>Levantamento Corpo</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3537,7 +3543,7 @@
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>000386</t>
+          <t>000370</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3560,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Levantamento Corpo</t>
+          <t>Chaparia Testeira + Saia + Canaletas</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3565,7 +3571,7 @@
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>000370</t>
+          <t>000371</t>
         </is>
       </c>
     </row>
@@ -3582,18 +3588,18 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Chaparia Testeira + Saia + Canaletas</t>
+          <t>Bdj Esquerda Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E115" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>000371</t>
+          <t>001441</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3616,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Tubo + Mão francesa (inferior)</t>
+          <t>Bdj Direita Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3621,7 +3627,7 @@
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>001441</t>
+          <t>001442</t>
         </is>
       </c>
     </row>
@@ -3638,18 +3644,18 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Bdj Direita Tubo + Mão francesa (inferior)</t>
+          <t>Bdj Esquerda Base Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E117" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>001442</t>
+          <t>001443</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3672,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Base Tubo + Mão francesa (inferior)</t>
+          <t>Bdj Direita Base Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3677,7 +3683,7 @@
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>001443</t>
+          <t>001444</t>
         </is>
       </c>
     </row>
@@ -3694,18 +3700,18 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Bdj Direita Base Tubo + Mão francesa (inferior)</t>
+          <t>Bdj Esquerda Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E119" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>001444</t>
+          <t>001445</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3728,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Tubo + Mão francesa (superior)</t>
+          <t>Bdj Direita Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3733,7 +3739,7 @@
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>001445</t>
+          <t>001446</t>
         </is>
       </c>
     </row>
@@ -3750,18 +3756,18 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Bdj Direita Tubo + Mão francesa (superior)</t>
+          <t>Bdj Esquerda Base Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E121" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>001446</t>
+          <t>001447</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3784,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Base Tubo + Mão francesa (superior)</t>
+          <t>Bdj Direita Base Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3789,7 +3795,7 @@
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>001447</t>
+          <t>001448</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3812,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Bdj Direita Base Tubo + Mão francesa (superior)</t>
+          <t>Aramado Toldo</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3817,7 +3823,7 @@
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>001448</t>
+          <t>000376</t>
         </is>
       </c>
     </row>
@@ -3834,7 +3840,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Aramado Toldo</t>
+          <t>Aramado Toldo + Chapa Fixação</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3845,7 +3851,7 @@
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>000376</t>
+          <t>000377</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3868,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Aramado Toldo + Chapa Fixação</t>
+          <t>Parachoque + Chapa 2,65</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3873,37 +3879,12 @@
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>000377</t>
+          <t>000378</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Parachoque + Chapa 2,65</t>
-        </is>
-      </c>
-      <c r="D126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E126" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F126" s="1" t="inlineStr">
-        <is>
-          <t>000378</t>
-        </is>
-      </c>
+      <c r="F126" s="1" t="n"/>
     </row>
     <row r="127">
       <c r="F127" s="1" t="n"/>
@@ -3946,9 +3927,6 @@
     </row>
     <row r="140">
       <c r="F140" s="1" t="n"/>
-    </row>
-    <row r="141">
-      <c r="F141" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>